<commit_message>
Clarify private-label MOQ and packaging RFQ requirements
</commit_message>
<xml_diff>
--- a/assets/downloads/huijia-dog-gear-rfq-template.xlsx
+++ b/assets/downloads/huijia-dog-gear-rfq-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Brief" sheetId="1" r:id="Rac6bb8f3c79e45f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Breakdown" sheetId="2" r:id="R4452dbed6af849b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Brief" sheetId="1" r:id="R49b8cc6943614783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Breakdown" sheetId="2" r:id="Re5d43d6203474d95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -647,7 +647,7 @@
       </x:c>
       <x:c r="B24" s="15"/>
       <x:c r="C24" s="16" t="str">
-        <x:v>Individual or set packaging, artwork, barcode and language.</x:v>
+        <x:v>Individual/set pack; material, finished pack dimensions, pieces per pack, artwork, barcode and language.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">

</xml_diff>